<commit_message>
style: fix tab clipping and update villa grid results
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-喇沙汇.xlsx
+++ b/files/九龙-九龙塘-喇沙汇.xlsx
@@ -197,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -206,6 +206,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -719,7 +722,7 @@
           <t>4+房</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="4" t="n">
         <v>5151</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -732,10 +735,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="5" t="n">
         <v>187910000</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="5" t="n">
         <v>36480</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -765,7 +768,7 @@
           <t>4+房</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>5291</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -778,10 +781,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="5" t="n">
         <v>208012000</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="5" t="n">
         <v>39314</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -811,7 +814,7 @@
           <t>4+房</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="4" t="n">
         <v>4799</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -824,10 +827,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="5" t="n">
         <v>166060000</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="5" t="n">
         <v>34603</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -857,7 +860,7 @@
           <t>4+房</t>
         </is>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="4" t="n">
         <v>4940</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -870,10 +873,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="5" t="n">
         <v>170430000</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="5" t="n">
         <v>34500</v>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -886,7 +889,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
@@ -908,111 +911,111 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>喇沙汇 销控网格图</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>总套数</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>在售 (Sale)</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>已定价未售</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>已售 (Sold)</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>暂停销售</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>待售 (Pending)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F3" s="17" t="inlineStr">
+      <c r="F3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>楼层</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>2&amp;3</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr"/>
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>A2 | 5291呎 (4+房)
 $20801万
@@ -1020,8 +1023,8 @@
 (暂停销售)</t>
         </is>
       </c>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr"/>
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>B2 | 5151呎 (4+房)
 $18791万
@@ -1031,12 +1034,12 @@
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>G&amp;1</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>A1 | 4940呎 (4+房)
 $17043万
@@ -1044,8 +1047,8 @@
 (暂停销售)</t>
         </is>
       </c>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr"/>
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>B1 | 4799呎 (4+房)
 $16606万
@@ -1053,13 +1056,13 @@
 (暂停销售)</t>
         </is>
       </c>
-      <c r="E6" s="19" t="n"/>
+      <c r="E6" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>